<commit_message>
Added (credible) pathways to csv. Ran code with 13 iterations.
</commit_message>
<xml_diff>
--- a/output/support/scores.xlsx
+++ b/output/support/scores.xlsx
@@ -452,1402 +452,1402 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>8798</v>
+        <v>42031</v>
       </c>
       <c r="B2" t="n">
-        <v>24.8227</v>
+        <v>28.4332</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>12.41135</v>
+        <v>14.2166</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>7038</v>
+        <v>74837</v>
       </c>
       <c r="B3" t="n">
-        <v>22.8009</v>
+        <v>28.4332</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>11.40045</v>
+        <v>14.2166</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3207</v>
+        <v>8669</v>
       </c>
       <c r="B4" t="n">
-        <v>22.8009</v>
+        <v>28.4332</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>11.40045</v>
+        <v>14.2166</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8050</v>
+        <v>3078</v>
       </c>
       <c r="B5" t="n">
-        <v>22.8009</v>
+        <v>24.6321</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>11.40045</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9621</v>
+        <v>74089</v>
       </c>
       <c r="B6" t="n">
-        <v>22.8009</v>
+        <v>24.6321</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>11.40045</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>14202</v>
+        <v>69246</v>
       </c>
       <c r="B7" t="n">
-        <v>21.2276</v>
+        <v>24.6321</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>10.6138</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6734</v>
+        <v>75660</v>
       </c>
       <c r="B8" t="n">
-        <v>21.2276</v>
+        <v>24.6321</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>10.6138</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8731</v>
+        <v>42854</v>
       </c>
       <c r="B9" t="n">
-        <v>21.2276</v>
+        <v>24.6321</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>10.6138</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1185</v>
+        <v>40271</v>
       </c>
       <c r="B10" t="n">
-        <v>21.2276</v>
+        <v>24.6321</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>10.6138</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5216</v>
+        <v>73077</v>
       </c>
       <c r="B11" t="n">
-        <v>19.8573</v>
+        <v>24.6321</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>9.928649999999999</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>21168</v>
+        <v>6909</v>
       </c>
       <c r="B12" t="n">
-        <v>19.8573</v>
+        <v>24.6321</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>9.928649999999999</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>1408</v>
+        <v>7921</v>
       </c>
       <c r="B13" t="n">
-        <v>19.8573</v>
+        <v>24.6321</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>9.928649999999999</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2924</v>
+        <v>9492</v>
       </c>
       <c r="B14" t="n">
-        <v>18.6533</v>
+        <v>24.6321</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>9.326650000000001</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2909</v>
+        <v>36440</v>
       </c>
       <c r="B15" t="n">
-        <v>18.6533</v>
+        <v>24.6321</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>9.326650000000001</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>7485</v>
+        <v>41283</v>
       </c>
       <c r="B16" t="n">
-        <v>18.6533</v>
+        <v>24.6321</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>9.326650000000001</v>
+        <v>12.31605</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1506</v>
+        <v>1056</v>
       </c>
       <c r="B17" t="n">
-        <v>18.6533</v>
+        <v>23.6672</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>9.326650000000001</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>781</v>
+        <v>74770</v>
       </c>
       <c r="B18" t="n">
-        <v>16.80278333333333</v>
+        <v>23.6672</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>8.401391666666667</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3152</v>
+        <v>47435</v>
       </c>
       <c r="B19" t="n">
-        <v>15.9631</v>
+        <v>23.6672</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>7.981550000000001</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>10197</v>
+        <v>72773</v>
       </c>
       <c r="B20" t="n">
-        <v>15.9631</v>
+        <v>23.6672</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>7.981550000000001</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>21975</v>
+        <v>39967</v>
       </c>
       <c r="B21" t="n">
-        <v>15.9225</v>
+        <v>23.6672</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>7.96125</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>23121</v>
+        <v>8602</v>
       </c>
       <c r="B22" t="n">
-        <v>15.9225</v>
+        <v>23.6672</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>7.96125</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>21098</v>
+        <v>80241</v>
       </c>
       <c r="B23" t="n">
-        <v>15.3925</v>
+        <v>23.6672</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>7.69625</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>12690</v>
+        <v>34418</v>
       </c>
       <c r="B24" t="n">
-        <v>14.7781</v>
+        <v>23.6672</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
       </c>
       <c r="D24" t="n">
-        <v>7.38905</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1008</v>
+        <v>6605</v>
       </c>
       <c r="B25" t="n">
-        <v>14.2776</v>
+        <v>23.6672</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
       </c>
       <c r="D25" t="n">
-        <v>7.1388</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>18794</v>
+        <v>67224</v>
       </c>
       <c r="B26" t="n">
-        <v>13.8833</v>
+        <v>23.6672</v>
       </c>
       <c r="C26" t="n">
         <v>0</v>
       </c>
       <c r="D26" t="n">
-        <v>6.94165</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>7961</v>
+        <v>41964</v>
       </c>
       <c r="B27" t="n">
-        <v>13.8833</v>
+        <v>23.6672</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>6.94165</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>22045</v>
+        <v>14073</v>
       </c>
       <c r="B28" t="n">
-        <v>13.5616</v>
+        <v>23.6672</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>6.7808</v>
+        <v>11.8336</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3376</v>
+        <v>38449</v>
       </c>
       <c r="B29" t="n">
-        <v>13.5616</v>
+        <v>22.7751</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>6.7808</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>16730</v>
+        <v>34641</v>
       </c>
       <c r="B30" t="n">
-        <v>13.5616</v>
+        <v>22.7751</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>6.7808</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4930</v>
+        <v>87207</v>
       </c>
       <c r="B31" t="n">
-        <v>13.5428</v>
+        <v>22.7751</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>6.7714</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>7168</v>
+        <v>54401</v>
       </c>
       <c r="B32" t="n">
-        <v>13.3676</v>
+        <v>22.7751</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>6.6838</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>7930</v>
+        <v>71255</v>
       </c>
       <c r="B33" t="n">
-        <v>13.0587</v>
+        <v>22.7751</v>
       </c>
       <c r="C33" t="n">
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>6.52935</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>9114</v>
+        <v>1279</v>
       </c>
       <c r="B34" t="n">
-        <v>12.8873</v>
+        <v>22.7751</v>
       </c>
       <c r="C34" t="n">
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>6.443650000000001</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>9525</v>
+        <v>67447</v>
       </c>
       <c r="B35" t="n">
-        <v>12.8873</v>
+        <v>22.7751</v>
       </c>
       <c r="C35" t="n">
         <v>0</v>
       </c>
       <c r="D35" t="n">
-        <v>6.443650000000001</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>4168</v>
+        <v>21039</v>
       </c>
       <c r="B36" t="n">
-        <v>12.8873</v>
+        <v>22.7751</v>
       </c>
       <c r="C36" t="n">
         <v>0</v>
       </c>
       <c r="D36" t="n">
-        <v>6.443650000000001</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>25631</v>
+        <v>5087</v>
       </c>
       <c r="B37" t="n">
-        <v>12.8873</v>
+        <v>22.7751</v>
       </c>
       <c r="C37" t="n">
         <v>0</v>
       </c>
       <c r="D37" t="n">
-        <v>6.443650000000001</v>
+        <v>11.38755</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>383</v>
+        <v>73524</v>
       </c>
       <c r="B38" t="n">
-        <v>12.8873</v>
+        <v>21.9478</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
       </c>
       <c r="D38" t="n">
-        <v>6.443650000000001</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>17024</v>
+        <v>1377</v>
       </c>
       <c r="B39" t="n">
-        <v>12.8873</v>
+        <v>21.9478</v>
       </c>
       <c r="C39" t="n">
         <v>0</v>
       </c>
       <c r="D39" t="n">
-        <v>6.443650000000001</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>14626</v>
+        <v>68963</v>
       </c>
       <c r="B40" t="n">
-        <v>12.8873</v>
+        <v>21.9478</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>6.443650000000001</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>11980</v>
+        <v>68948</v>
       </c>
       <c r="B41" t="n">
-        <v>12.8873</v>
+        <v>21.9478</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>6.443650000000001</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>7995</v>
+        <v>67545</v>
       </c>
       <c r="B42" t="n">
-        <v>12.8873</v>
+        <v>21.9478</v>
       </c>
       <c r="C42" t="n">
         <v>0</v>
       </c>
       <c r="D42" t="n">
-        <v>6.443650000000001</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>21226</v>
+        <v>40718</v>
       </c>
       <c r="B43" t="n">
-        <v>12.8873</v>
+        <v>21.9478</v>
       </c>
       <c r="C43" t="n">
         <v>0</v>
       </c>
       <c r="D43" t="n">
-        <v>6.443650000000001</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>9700</v>
+        <v>36142</v>
       </c>
       <c r="B44" t="n">
-        <v>12.8873</v>
+        <v>21.9478</v>
       </c>
       <c r="C44" t="n">
         <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>6.443650000000001</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>19467</v>
+        <v>36157</v>
       </c>
       <c r="B45" t="n">
-        <v>12.8873</v>
+        <v>21.9478</v>
       </c>
       <c r="C45" t="n">
         <v>0</v>
       </c>
       <c r="D45" t="n">
-        <v>6.443650000000001</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>17046</v>
+        <v>7356</v>
       </c>
       <c r="B46" t="n">
-        <v>12.8725</v>
+        <v>21.9478</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
       </c>
       <c r="D46" t="n">
-        <v>6.43625</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>13856</v>
+        <v>2795</v>
       </c>
       <c r="B47" t="n">
-        <v>12.2241</v>
+        <v>21.9478</v>
       </c>
       <c r="C47" t="n">
         <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>6.11205</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>13374</v>
+        <v>34739</v>
       </c>
       <c r="B48" t="n">
-        <v>12.2241</v>
+        <v>21.9478</v>
       </c>
       <c r="C48" t="n">
         <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>6.11205</v>
+        <v>10.9739</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>21436</v>
+        <v>34014</v>
       </c>
       <c r="B49" t="n">
-        <v>12.091</v>
+        <v>20.83746666666667</v>
       </c>
       <c r="C49" t="n">
         <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>6.0455</v>
+        <v>10.41873333333333</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2848</v>
+        <v>66820</v>
       </c>
       <c r="B50" t="n">
-        <v>12.091</v>
+        <v>20.83746666666667</v>
       </c>
       <c r="C50" t="n">
         <v>0</v>
       </c>
       <c r="D50" t="n">
-        <v>6.0455</v>
+        <v>10.41873333333333</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>18275</v>
+        <v>652</v>
       </c>
       <c r="B51" t="n">
-        <v>12.0605</v>
+        <v>20.83746666666667</v>
       </c>
       <c r="C51" t="n">
         <v>0</v>
       </c>
       <c r="D51" t="n">
-        <v>6.03025</v>
+        <v>10.41873333333333</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>12094</v>
+        <v>98932</v>
       </c>
       <c r="B52" t="n">
         <v>0</v>
       </c>
       <c r="C52" t="n">
-        <v>0.8988950252532959</v>
+        <v>0.9436925649642944</v>
       </c>
       <c r="D52" t="n">
-        <v>0.2633110273872588</v>
+        <v>0.2572423278314001</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>315</v>
+        <v>32764</v>
       </c>
       <c r="B53" t="n">
         <v>0</v>
       </c>
       <c r="C53" t="n">
-        <v>0.8995209634304047</v>
+        <v>0.9436925649642944</v>
       </c>
       <c r="D53" t="n">
-        <v>0.2632242600245034</v>
+        <v>0.2572423278314001</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>15965</v>
+        <v>33169</v>
       </c>
       <c r="B54" t="n">
         <v>0</v>
       </c>
       <c r="C54" t="n">
-        <v>0.9020004272460938</v>
+        <v>0.944710373878479</v>
       </c>
       <c r="D54" t="n">
-        <v>0.2628811186567134</v>
+        <v>0.2571076941410114</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>18097</v>
+        <v>99337</v>
       </c>
       <c r="B55" t="n">
         <v>0</v>
       </c>
       <c r="C55" t="n">
-        <v>0.9020424783229828</v>
+        <v>0.944710373878479</v>
       </c>
       <c r="D55" t="n">
-        <v>0.2628753067811853</v>
+        <v>0.2571076941410114</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>1974</v>
+        <v>31820</v>
       </c>
       <c r="B56" t="n">
         <v>0</v>
       </c>
       <c r="C56" t="n">
-        <v>0.9023942947387695</v>
+        <v>0.9447717666625977</v>
       </c>
       <c r="D56" t="n">
-        <v>0.2628266923333358</v>
+        <v>0.2570995777350495</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>12756</v>
+        <v>97988</v>
       </c>
       <c r="B57" t="n">
         <v>0</v>
       </c>
       <c r="C57" t="n">
-        <v>0.9029656648635864</v>
+        <v>0.9447717666625977</v>
       </c>
       <c r="D57" t="n">
-        <v>0.2627477779720436</v>
+        <v>0.2570995777350495</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>17243</v>
+        <v>12075</v>
       </c>
       <c r="B58" t="n">
         <v>0</v>
       </c>
       <c r="C58" t="n">
-        <v>0.9031985998153687</v>
+        <v>0.9460305571556091</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2627156199297885</v>
+        <v>0.2569332727903403</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>14790</v>
+        <v>78243</v>
       </c>
       <c r="B59" t="n">
         <v>0</v>
       </c>
       <c r="C59" t="n">
-        <v>0.9039535522460938</v>
+        <v>0.9460306167602539</v>
       </c>
       <c r="D59" t="n">
-        <v>0.2626114483781131</v>
+        <v>0.2569332649207742</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>11250</v>
+        <v>99281</v>
       </c>
       <c r="B60" t="n">
         <v>0</v>
       </c>
       <c r="C60" t="n">
-        <v>0.9044677019119263</v>
+        <v>0.9470149278640747</v>
       </c>
       <c r="D60" t="n">
-        <v>0.2625405510936425</v>
+        <v>0.2568033726112788</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>5203</v>
+        <v>33113</v>
       </c>
       <c r="B61" t="n">
         <v>0</v>
       </c>
       <c r="C61" t="n">
-        <v>0.9044732451438904</v>
+        <v>0.9470149278640747</v>
       </c>
       <c r="D61" t="n">
-        <v>0.2625397869331701</v>
+        <v>0.2568033726112788</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>10539</v>
+        <v>98659</v>
       </c>
       <c r="B62" t="n">
         <v>0</v>
       </c>
       <c r="C62" t="n">
-        <v>0.905234232544899</v>
+        <v>0.9518953561782837</v>
       </c>
       <c r="D62" t="n">
-        <v>0.2624349234645704</v>
+        <v>0.2561612734091318</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>11860</v>
+        <v>32491</v>
       </c>
       <c r="B63" t="n">
         <v>0</v>
       </c>
       <c r="C63" t="n">
-        <v>0.9052505493164062</v>
+        <v>0.9518953561782837</v>
       </c>
       <c r="D63" t="n">
-        <v>0.2624326759435379</v>
+        <v>0.2561612734091318</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>14704</v>
+        <v>32842</v>
       </c>
       <c r="B64" t="n">
         <v>0</v>
       </c>
       <c r="C64" t="n">
-        <v>0.9056225717067719</v>
+        <v>0.9562438130378723</v>
       </c>
       <c r="D64" t="n">
-        <v>0.2623814429067004</v>
+        <v>0.2555918626643703</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>17269</v>
+        <v>99010</v>
       </c>
       <c r="B65" t="n">
         <v>0</v>
       </c>
       <c r="C65" t="n">
-        <v>0.906856432557106</v>
+        <v>0.9562438130378723</v>
       </c>
       <c r="D65" t="n">
-        <v>0.2622116649492574</v>
+        <v>0.2555918626643703</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>13147</v>
+        <v>31414</v>
       </c>
       <c r="B66" t="n">
         <v>0</v>
       </c>
       <c r="C66" t="n">
-        <v>0.9072015881538391</v>
+        <v>0.9575133323669434</v>
       </c>
       <c r="D66" t="n">
-        <v>0.2621642112221589</v>
+        <v>0.2554261019491606</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>4455</v>
+        <v>97582</v>
       </c>
       <c r="B67" t="n">
         <v>0</v>
       </c>
       <c r="C67" t="n">
-        <v>0.9072189182043076</v>
+        <v>0.9575133323669434</v>
       </c>
       <c r="D67" t="n">
-        <v>0.2621618290525148</v>
+        <v>0.2554261019491606</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>26999</v>
+        <v>99131</v>
       </c>
       <c r="B68" t="n">
         <v>0</v>
       </c>
       <c r="C68" t="n">
-        <v>0.9076013565063477</v>
+        <v>0.9576199173927307</v>
       </c>
       <c r="D68" t="n">
-        <v>0.2621092705216559</v>
+        <v>0.2554121949606686</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>5226</v>
+        <v>32055</v>
       </c>
       <c r="B69" t="n">
         <v>0</v>
       </c>
       <c r="C69" t="n">
-        <v>0.9076150059700012</v>
+        <v>0.9576199173927307</v>
       </c>
       <c r="D69" t="n">
-        <v>0.2621073950641081</v>
+        <v>0.2554121949606686</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>14251</v>
+        <v>98223</v>
       </c>
       <c r="B70" t="n">
         <v>0</v>
       </c>
       <c r="C70" t="n">
-        <v>0.9079282283782959</v>
+        <v>0.9576199173927307</v>
       </c>
       <c r="D70" t="n">
-        <v>0.2620643651910276</v>
+        <v>0.2554121949606686</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>13100</v>
+        <v>32963</v>
       </c>
       <c r="B71" t="n">
         <v>0</v>
       </c>
       <c r="C71" t="n">
-        <v>0.9079800844192505</v>
+        <v>0.9576199173927307</v>
       </c>
       <c r="D71" t="n">
-        <v>0.2620572426740972</v>
+        <v>0.2554121949606686</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>3085</v>
+        <v>32964</v>
       </c>
       <c r="B72" t="n">
         <v>0</v>
       </c>
       <c r="C72" t="n">
-        <v>0.9084427356719971</v>
+        <v>0.9578140258789063</v>
       </c>
       <c r="D72" t="n">
-        <v>0.2619937138558894</v>
+        <v>0.2553868719862393</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>13442</v>
+        <v>99132</v>
       </c>
       <c r="B73" t="n">
         <v>0</v>
       </c>
       <c r="C73" t="n">
-        <v>0.908580482006073</v>
+        <v>0.9578140258789063</v>
       </c>
       <c r="D73" t="n">
-        <v>0.261974805209398</v>
+        <v>0.2553868719862393</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>16205</v>
+        <v>32056</v>
       </c>
       <c r="B74" t="n">
         <v>0</v>
       </c>
       <c r="C74" t="n">
-        <v>0.9086835086345673</v>
+        <v>0.9578140258789063</v>
       </c>
       <c r="D74" t="n">
-        <v>0.2619606643731572</v>
+        <v>0.2553868719862393</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>21782</v>
+        <v>98224</v>
       </c>
       <c r="B75" t="n">
         <v>0</v>
       </c>
       <c r="C75" t="n">
-        <v>0.9090400040149689</v>
+        <v>0.9578140258789063</v>
       </c>
       <c r="D75" t="n">
-        <v>0.2619117456671586</v>
+        <v>0.2553868719862393</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>14463</v>
+        <v>97309</v>
       </c>
       <c r="B76" t="n">
         <v>0</v>
       </c>
       <c r="C76" t="n">
-        <v>0.9099763184785843</v>
+        <v>0.9580875039100647</v>
       </c>
       <c r="D76" t="n">
-        <v>0.2617833504858748</v>
+        <v>0.2553512031518307</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>4653</v>
+        <v>31141</v>
       </c>
       <c r="B77" t="n">
         <v>0</v>
       </c>
       <c r="C77" t="n">
-        <v>0.9101221164067587</v>
+        <v>0.9580875039100647</v>
       </c>
       <c r="D77" t="n">
-        <v>0.2617633687947548</v>
+        <v>0.2553512031518307</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>13638</v>
+        <v>32448</v>
       </c>
       <c r="B78" t="n">
         <v>0</v>
       </c>
       <c r="C78" t="n">
-        <v>0.9104804793993632</v>
+        <v>0.9581061204274496</v>
       </c>
       <c r="D78" t="n">
-        <v>0.2617142678983013</v>
+        <v>0.2553487754232908</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>15886</v>
+        <v>98616</v>
       </c>
       <c r="B79" t="n">
         <v>0</v>
       </c>
       <c r="C79" t="n">
-        <v>0.9106599092483521</v>
+        <v>0.9581061204274496</v>
       </c>
       <c r="D79" t="n">
-        <v>0.2616896903419607</v>
+        <v>0.2553487754232908</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>4961</v>
+        <v>32797</v>
       </c>
       <c r="B80" t="n">
         <v>0</v>
       </c>
       <c r="C80" t="n">
-        <v>0.9115528225898742</v>
+        <v>0.9581381678581238</v>
       </c>
       <c r="D80" t="n">
-        <v>0.2615674513888521</v>
+        <v>0.2553445963146291</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>5114</v>
+        <v>98965</v>
       </c>
       <c r="B81" t="n">
         <v>0</v>
       </c>
       <c r="C81" t="n">
-        <v>0.9117672840754191</v>
+        <v>0.9581381678581238</v>
       </c>
       <c r="D81" t="n">
-        <v>0.2615381088299213</v>
+        <v>0.2553445963146291</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>17377</v>
+        <v>97205</v>
       </c>
       <c r="B82" t="n">
         <v>0</v>
       </c>
       <c r="C82" t="n">
-        <v>0.9118037819862366</v>
+        <v>0.9586269855499268</v>
       </c>
       <c r="D82" t="n">
-        <v>0.2615331158517394</v>
+        <v>0.2552808695524095</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>11873</v>
+        <v>31037</v>
       </c>
       <c r="B83" t="n">
         <v>0</v>
       </c>
       <c r="C83" t="n">
-        <v>0.9126194715499878</v>
+        <v>0.9586269855499268</v>
       </c>
       <c r="D83" t="n">
-        <v>0.2614215778085746</v>
+        <v>0.2552808695524095</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>16130</v>
+        <v>31537</v>
       </c>
       <c r="B84" t="n">
         <v>0</v>
       </c>
       <c r="C84" t="n">
-        <v>0.9132238427797953</v>
+        <v>0.9596409797668457</v>
       </c>
       <c r="D84" t="n">
-        <v>0.2613389969432595</v>
+        <v>0.2551487773334323</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1968</v>
+        <v>97705</v>
       </c>
       <c r="B85" t="n">
         <v>0</v>
       </c>
       <c r="C85" t="n">
-        <v>0.9138243198394775</v>
+        <v>0.9596409797668457</v>
       </c>
       <c r="D85" t="n">
-        <v>0.2612569998284574</v>
+        <v>0.2551487773334323</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>29079</v>
+        <v>83264</v>
       </c>
       <c r="B86" t="n">
         <v>0</v>
       </c>
       <c r="C86" t="n">
-        <v>0.9138715147972107</v>
+        <v>0.9597234427928925</v>
       </c>
       <c r="D86" t="n">
-        <v>0.2612505573828862</v>
+        <v>0.2551380409510369</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>7855</v>
+        <v>17096</v>
       </c>
       <c r="B87" t="n">
         <v>0</v>
       </c>
       <c r="C87" t="n">
-        <v>0.9144208331902822</v>
+        <v>0.9597234576940536</v>
       </c>
       <c r="D87" t="n">
-        <v>0.2611755949013447</v>
+        <v>0.2551380390110422</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>10524</v>
+        <v>31810</v>
       </c>
       <c r="B88" t="n">
         <v>0</v>
       </c>
       <c r="C88" t="n">
-        <v>0.9147552102804184</v>
+        <v>0.9600329756736755</v>
       </c>
       <c r="D88" t="n">
-        <v>0.2611299853451107</v>
+        <v>0.2550977489693238</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>13384</v>
+        <v>97978</v>
       </c>
       <c r="B89" t="n">
         <v>0</v>
       </c>
       <c r="C89" t="n">
-        <v>0.9150511920452118</v>
+        <v>0.9600329756736755</v>
       </c>
       <c r="D89" t="n">
-        <v>0.2610896262600774</v>
+        <v>0.2550977489693238</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>17256</v>
+        <v>17093</v>
       </c>
       <c r="B90" t="n">
         <v>0</v>
       </c>
       <c r="C90" t="n">
-        <v>0.9152307748794556</v>
+        <v>0.9600952863693237</v>
       </c>
       <c r="D90" t="n">
-        <v>0.2610651450248704</v>
+        <v>0.2550896395073465</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>13990</v>
+        <v>83261</v>
       </c>
       <c r="B91" t="n">
         <v>0</v>
       </c>
       <c r="C91" t="n">
-        <v>0.9154833257198334</v>
+        <v>0.9600952863693237</v>
       </c>
       <c r="D91" t="n">
-        <v>0.261030724353657</v>
+        <v>0.2550896395073465</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>13782</v>
+        <v>32089</v>
       </c>
       <c r="B92" t="n">
         <v>0</v>
       </c>
       <c r="C92" t="n">
-        <v>0.9158063769340515</v>
+        <v>0.9602213144302368</v>
       </c>
       <c r="D92" t="n">
-        <v>0.2609867082706823</v>
+        <v>0.2550732390874605</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>15737</v>
+        <v>32997</v>
       </c>
       <c r="B93" t="n">
         <v>0</v>
       </c>
       <c r="C93" t="n">
-        <v>0.9161118268966675</v>
+        <v>0.9602213144302368</v>
       </c>
       <c r="D93" t="n">
-        <v>0.2609451040286095</v>
+        <v>0.2550732390874605</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>12204</v>
+        <v>98257</v>
       </c>
       <c r="B94" t="n">
         <v>0</v>
       </c>
       <c r="C94" t="n">
-        <v>0.9174277037382126</v>
+        <v>0.9602213144302368</v>
       </c>
       <c r="D94" t="n">
-        <v>0.2607660247242705</v>
+        <v>0.2550732390874605</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>15638</v>
+        <v>99165</v>
       </c>
       <c r="B95" t="n">
         <v>0</v>
       </c>
       <c r="C95" t="n">
-        <v>0.917534863948822</v>
+        <v>0.9602213144302368</v>
       </c>
       <c r="D95" t="n">
-        <v>0.2607514519816025</v>
+        <v>0.2550732390874605</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>11256</v>
+        <v>30985</v>
       </c>
       <c r="B96" t="n">
         <v>0</v>
       </c>
       <c r="C96" t="n">
-        <v>0.9178102115790049</v>
+        <v>0.9605373263359069</v>
       </c>
       <c r="D96" t="n">
-        <v>0.2607140148598601</v>
+        <v>0.2550321247565643</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>15649</v>
+        <v>97153</v>
       </c>
       <c r="B97" t="n">
         <v>0</v>
       </c>
       <c r="C97" t="n">
-        <v>0.918267160654068</v>
+        <v>0.9605373263359069</v>
       </c>
       <c r="D97" t="n">
-        <v>0.2606519103572184</v>
+        <v>0.2550321247565643</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>13204</v>
+        <v>32913</v>
       </c>
       <c r="B98" t="n">
         <v>0</v>
       </c>
       <c r="C98" t="n">
-        <v>0.9182976722717285</v>
+        <v>0.9605796784162521</v>
       </c>
       <c r="D98" t="n">
-        <v>0.2606477645400461</v>
+        <v>0.255026615599677</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>16128</v>
+        <v>99081</v>
       </c>
       <c r="B99" t="n">
         <v>0</v>
       </c>
       <c r="C99" t="n">
-        <v>0.9185062646865845</v>
+        <v>0.9605796784162521</v>
       </c>
       <c r="D99" t="n">
-        <v>0.2606194252285552</v>
+        <v>0.255026615599677</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>16348</v>
+        <v>31811</v>
       </c>
       <c r="B100" t="n">
         <v>0</v>
       </c>
       <c r="C100" t="n">
-        <v>0.9185771703720093</v>
+        <v>0.9610133469104767</v>
       </c>
       <c r="D100" t="n">
-        <v>0.2606097934038539</v>
+        <v>0.2549702177130698</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>23651</v>
+        <v>97979</v>
       </c>
       <c r="B101" t="n">
         <v>0</v>
       </c>
       <c r="C101" t="n">
-        <v>0.9187114040056864</v>
+        <v>0.9610133469104767</v>
       </c>
       <c r="D101" t="n">
-        <v>0.2605915610634054</v>
+        <v>0.2549702177130698</v>
       </c>
     </row>
   </sheetData>

</xml_diff>